<commit_message>
feat: buatkan draf IOM resmi PT KAB No. 005/MKT/KAB/GREN/IX/2026 dan perbarui master register
</commit_message>
<xml_diff>
--- a/00_STANDAR_DAN_REGULASI/BUKU_AGENDA_DAN_REGISTER_NOMOR_SURAT.xlsx
+++ b/00_STANDAR_DAN_REGULASI/BUKU_AGENDA_DAN_REGISTER_NOMOR_SURAT.xlsx
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M28"/>
+  <dimension ref="A1:M29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -562,7 +562,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Terakhir Diperbarui: 21 September 2026 | Total Terdaftar: 23 Berkas</t>
+          <t>Terakhir Diperbarui: 21 September 2026 | Total Terdaftar: 24 Berkas</t>
         </is>
       </c>
     </row>
@@ -2126,6 +2126,71 @@
       <c r="M28" s="6" t="inlineStr">
         <is>
           <t>01_GREN_PROPERTYKOST/06_SPK_Dan_Kontrak/PKS_PT_Kenzo_Anatha_Bumi_Aswar_Anas_Digital_Marketing_Meta_Ads.docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>REG-2026-0024</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>005/MKT/KAB/GREN/IX/2026</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>GREN</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>KAB</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>MKT</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>IOM</t>
+        </is>
+      </c>
+      <c r="I29" s="9" t="inlineStr">
+        <is>
+          <t>Kebijakan Program Penjualan &amp; Aktivasi Marketing Kuartal IV 2026</t>
+        </is>
+      </c>
+      <c r="J29" s="9" t="inlineStr">
+        <is>
+          <t>Divisi Sales &amp; Marketing GREN Propertykost</t>
+        </is>
+      </c>
+      <c r="K29" s="9" t="inlineStr">
+        <is>
+          <t>Divisi Marketing Communication</t>
+        </is>
+      </c>
+      <c r="L29" s="7" t="inlineStr">
+        <is>
+          <t>DITERBITKAN</t>
+        </is>
+      </c>
+      <c r="M29" s="9" t="inlineStr">
+        <is>
+          <t>01_GREN_PROPERTYKOST/03_Internal_Office_Memo_IOM/005_MKT_KAB_GREN_IX_2026_IOM_Program_Penjualan_Sales.docx</t>
         </is>
       </c>
     </row>
@@ -2860,7 +2925,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Total Dokumen Terdaftar: 23 Berkas</t>
+          <t>Total Dokumen Terdaftar: 24 Berkas</t>
         </is>
       </c>
     </row>
@@ -2906,11 +2971,11 @@
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>30.4%</t>
+          <t>33.3%</t>
         </is>
       </c>
     </row>
@@ -2933,7 +2998,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>47.8%</t>
+          <t>45.8%</t>
         </is>
       </c>
     </row>
@@ -3002,7 +3067,7 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>4.3%</t>
+          <t>4.2%</t>
         </is>
       </c>
     </row>
@@ -3048,7 +3113,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>17.4%</t>
+          <t>16.7%</t>
         </is>
       </c>
     </row>
@@ -3065,7 +3130,7 @@
         </is>
       </c>
       <c r="D12" s="14" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
refactor: tetapkan nomor tunggal resmi IOM KAB menjadi 004/MKT/KAB/GREN/IX/2026 dan hapus draf nomor 005
</commit_message>
<xml_diff>
--- a/00_STANDAR_DAN_REGULASI/BUKU_AGENDA_DAN_REGISTER_NOMOR_SURAT.xlsx
+++ b/00_STANDAR_DAN_REGULASI/BUKU_AGENDA_DAN_REGISTER_NOMOR_SURAT.xlsx
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M29"/>
+  <dimension ref="A1:M28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -562,7 +562,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Terakhir Diperbarui: 21 September 2026 | Total Terdaftar: 24 Berkas</t>
+          <t>Terakhir Diperbarui: 21 September 2026 | Total Terdaftar: 23 Berkas</t>
         </is>
       </c>
     </row>
@@ -965,27 +965,27 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>REG-2026-0006</t>
+          <t>REG-2026-0007</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>004/MKT/KAB/GREN/IX/2026</t>
+          <t>002/MKT/YPL/VI/2026</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>GREN</t>
+          <t>CORP</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>KAB</t>
+          <t>YPL</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -995,32 +995,32 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>SURAT</t>
+          <t>IOM</t>
         </is>
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>Permohonan Kerjasama Tenant Kampus</t>
+          <t>Skema Closing Fee (CF) Sales, SPV, &amp; SM Periode Juni - Desember 2026</t>
         </is>
       </c>
       <c r="J11" s="9" t="inlineStr">
         <is>
-          <t>Rektorat Unpad</t>
+          <t>Seluruh Rekan Sales &amp; Agent</t>
         </is>
       </c>
       <c r="K11" s="9" t="inlineStr">
         <is>
-          <t>Divisi MKT</t>
+          <t>Divisi Marketing Communication / Management</t>
         </is>
       </c>
       <c r="L11" s="7" t="inlineStr">
         <is>
-          <t>DITERBITKAN</t>
+          <t>TERARSIP</t>
         </is>
       </c>
       <c r="M11" s="9" t="inlineStr">
         <is>
-          <t>01_GREN_PROPERTYKOST\01_Surat_Keluar/004_MKT_KAB_GREN_IX_2026_Permohonan_Kerjasama_Tenant_Kampus.docx</t>
+          <t>07_CORPORATE_YANPROLAND_HOLDING/03_Internal_Office_Memo_Holding/002_MKT_YPL_VI_2026_IOM_Skema_Closing_Fee_Sales_Juni_Desember_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1030,17 +1030,17 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>REG-2026-0007</t>
+          <t>REG-2026-0008</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>002/MKT/YPL/VI/2026</t>
+          <t>004/MKT/YPL/VI/2026</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>Skema Closing Fee (CF) Sales, SPV, &amp; SM Periode Juni - Desember 2026</t>
+          <t>Skema Komisi (Fee) Sales &amp; Promo Spesial Juni - Juli 2026</t>
         </is>
       </c>
       <c r="J12" s="6" t="inlineStr">
@@ -1085,7 +1085,7 @@
       </c>
       <c r="M12" s="6" t="inlineStr">
         <is>
-          <t>07_CORPORATE_YANPROLAND_HOLDING/03_Internal_Office_Memo_Holding/002_MKT_YPL_VI_2026_IOM_Skema_Closing_Fee_Sales_Juni_Desember_2026.pdf</t>
+          <t>07_CORPORATE_YANPROLAND_HOLDING/03_Internal_Office_Memo_Holding/004_MKT_YPL_VI_2026_IOM_Skema_Komisi_Sales_Juni_Juli_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1095,27 +1095,27 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>REG-2026-0008</t>
+          <t>REG-2026-0009</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>004/MKT/YPL/VI/2026</t>
+          <t>002/PP/GREN-PKJ/2026</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>CORP</t>
+          <t>GREN</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>YPL</t>
+          <t>KAB</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1125,22 +1125,22 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>IOM</t>
+          <t>SURAT_KELUAR</t>
         </is>
       </c>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t>Skema Komisi (Fee) Sales &amp; Promo Spesial Juni - Juli 2026</t>
+          <t>Permohonan Izin Open Table &amp; Distribusi Brosur SESKO TNI</t>
         </is>
       </c>
       <c r="J13" s="9" t="inlineStr">
         <is>
-          <t>Seluruh Rekan Sales &amp; Agent</t>
+          <t>KAPRIM SESKO TNI Bandung</t>
         </is>
       </c>
       <c r="K13" s="9" t="inlineStr">
         <is>
-          <t>Divisi Marketing Communication / Management</t>
+          <t>Tim Marketing GREN Propertykost</t>
         </is>
       </c>
       <c r="L13" s="7" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="M13" s="9" t="inlineStr">
         <is>
-          <t>07_CORPORATE_YANPROLAND_HOLDING/03_Internal_Office_Memo_Holding/004_MKT_YPL_VI_2026_IOM_Skema_Komisi_Sales_Juni_Juli_2026.pdf</t>
+          <t>01_GREN_PROPERTYKOST/01_Surat_Keluar/002_PP_GREN_PKJ_2026_Permohonan_Open_Table_SESKO_TNI_Bandung.pdf</t>
         </is>
       </c>
     </row>
@@ -1160,52 +1160,52 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>REG-2026-0009</t>
+          <t>REG-2026-0010</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>002/PP/GREN-PKJ/2026</t>
+          <t>200/UN31.25/KM/2026</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>GREN</t>
+          <t>FNA</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>KAB</t>
+          <t>NAI</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>MKT</t>
+          <t>EXT</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>SURAT_KELUAR</t>
+          <t>SURAT_MASUK</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>Permohonan Izin Open Table &amp; Distribusi Brosur SESKO TNI</t>
+          <t>Surat Keterangan Mahasiswa Aktif UT Padang a.n. Nugi Fathul Falah</t>
         </is>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>KAPRIM SESKO TNI Bandung</t>
+          <t>Nugi Fathul Falah</t>
         </is>
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>Tim Marketing GREN Propertykost</t>
+          <t>Kepala UPBJJ-UT Padang</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="M14" s="6" t="inlineStr">
         <is>
-          <t>01_GREN_PROPERTYKOST/01_Surat_Keluar/002_PP_GREN_PKJ_2026_Permohonan_Open_Table_SESKO_TNI_Bandung.pdf</t>
+          <t>05_FREELANCE_NUGI_AI_STUDIO/02_Surat_Masuk/200_UN31_25_KM_2026_Surat_Keterangan_Mahasiswa_Aktif_UT_Nugi_Fathul_Falah.pdf</t>
         </is>
       </c>
     </row>
@@ -1225,52 +1225,52 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>REG-2026-0010</t>
+          <t>REG-2026-0011</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>200/UN31.25/KM/2026</t>
+          <t>001/OT/YPL/03/IX/2026</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>FNA</t>
+          <t>HJA</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>NAI</t>
+          <t>YPL</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>EXT</t>
+          <t>MKT</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>SURAT_MASUK</t>
+          <t>UNDANGAN</t>
         </is>
       </c>
       <c r="I15" s="9" t="inlineStr">
         <is>
-          <t>Surat Keterangan Mahasiswa Aktif UT Padang a.n. Nugi Fathul Falah</t>
+          <t>Undangan Open Table Jatihandap Asri di Dapur Hawu (Pak Rhendy)</t>
         </is>
       </c>
       <c r="J15" s="9" t="inlineStr">
         <is>
-          <t>Nugi Fathul Falah</t>
+          <t>Pak Rhendy</t>
         </is>
       </c>
       <c r="K15" s="9" t="inlineStr">
         <is>
-          <t>Kepala UPBJJ-UT Padang</t>
+          <t>Tim Marketing Jatihandap Asri</t>
         </is>
       </c>
       <c r="L15" s="7" t="inlineStr">
@@ -1280,7 +1280,7 @@
       </c>
       <c r="M15" s="9" t="inlineStr">
         <is>
-          <t>05_FREELANCE_NUGI_AI_STUDIO/02_Surat_Masuk/200_UN31_25_KM_2026_Surat_Keterangan_Mahasiswa_Aktif_UT_Nugi_Fathul_Falah.pdf</t>
+          <t>02_HUNIAN_ASRI_JATIHANDAP/01_Surat_Keluar/001_OT_YPL_03_IX_2026_Undangan_Open_Table_Pak_Rhendy.pdf</t>
         </is>
       </c>
     </row>
@@ -1290,12 +1290,12 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>REG-2026-0011</t>
+          <t>REG-2026-0012</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>001/OT/YPL/03/IX/2026</t>
+          <t>002/OT/YPL/03/IX/2026</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -1325,12 +1325,12 @@
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>Undangan Open Table Jatihandap Asri di Dapur Hawu (Pak Rhendy)</t>
+          <t>Undangan Open Table Jatihandap Asri di Dapur Hawu (Bu Euis)</t>
         </is>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>Pak Rhendy</t>
+          <t>Bu Euis</t>
         </is>
       </c>
       <c r="K16" s="6" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="M16" s="6" t="inlineStr">
         <is>
-          <t>02_HUNIAN_ASRI_JATIHANDAP/01_Surat_Keluar/001_OT_YPL_03_IX_2026_Undangan_Open_Table_Pak_Rhendy.pdf</t>
+          <t>02_HUNIAN_ASRI_JATIHANDAP/01_Surat_Keluar/002_OT_YPL_03_IX_2026_Undangan_Open_Table_Bu_Euis.pdf</t>
         </is>
       </c>
     </row>
@@ -1355,12 +1355,12 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>REG-2026-0012</t>
+          <t>REG-2026-0013</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>002/OT/YPL/03/IX/2026</t>
+          <t>003/OT/YPL/03/IX/2026</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
@@ -1390,12 +1390,12 @@
       </c>
       <c r="I17" s="9" t="inlineStr">
         <is>
-          <t>Undangan Open Table Jatihandap Asri di Dapur Hawu (Bu Euis)</t>
+          <t>Undangan Open Table Jatihandap Asri di Dapur Hawu (Ibu Haji Deden)</t>
         </is>
       </c>
       <c r="J17" s="9" t="inlineStr">
         <is>
-          <t>Bu Euis</t>
+          <t>Ibu Haji Deden</t>
         </is>
       </c>
       <c r="K17" s="9" t="inlineStr">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="M17" s="9" t="inlineStr">
         <is>
-          <t>02_HUNIAN_ASRI_JATIHANDAP/01_Surat_Keluar/002_OT_YPL_03_IX_2026_Undangan_Open_Table_Bu_Euis.pdf</t>
+          <t>02_HUNIAN_ASRI_JATIHANDAP/01_Surat_Keluar/003_OT_YPL_03_IX_2026_Undangan_Open_Table_Ibu_Haji_Deden.pdf</t>
         </is>
       </c>
     </row>
@@ -1420,12 +1420,12 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>REG-2026-0013</t>
+          <t>REG-2026-0014</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>003/OT/YPL/03/IX/2026</t>
+          <t>004/OT/YPL/03/IX/2026</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -1455,12 +1455,12 @@
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>Undangan Open Table Jatihandap Asri di Dapur Hawu (Ibu Haji Deden)</t>
+          <t>Undangan Open Table Jatihandap Asri di Dapur Hawu (Pak Fasha)</t>
         </is>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>Ibu Haji Deden</t>
+          <t>Pak Fasha</t>
         </is>
       </c>
       <c r="K18" s="6" t="inlineStr">
@@ -1475,7 +1475,7 @@
       </c>
       <c r="M18" s="6" t="inlineStr">
         <is>
-          <t>02_HUNIAN_ASRI_JATIHANDAP/01_Surat_Keluar/003_OT_YPL_03_IX_2026_Undangan_Open_Table_Ibu_Haji_Deden.pdf</t>
+          <t>02_HUNIAN_ASRI_JATIHANDAP/01_Surat_Keluar/004_OT_YPL_03_IX_2026_Undangan_Open_Table_Pak_Fasha.pdf</t>
         </is>
       </c>
     </row>
@@ -1485,12 +1485,12 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>REG-2026-0014</t>
+          <t>REG-2026-0015</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>004/OT/YPL/03/IX/2026</t>
+          <t>005/OT/YPL/03/IX/2026</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
@@ -1520,12 +1520,12 @@
       </c>
       <c r="I19" s="9" t="inlineStr">
         <is>
-          <t>Undangan Open Table Jatihandap Asri di Dapur Hawu (Pak Fasha)</t>
+          <t>Undangan Open Table Jatihandap Asri di Dapur Hawu (Ibu Re)</t>
         </is>
       </c>
       <c r="J19" s="9" t="inlineStr">
         <is>
-          <t>Pak Fasha</t>
+          <t>Ibu Re</t>
         </is>
       </c>
       <c r="K19" s="9" t="inlineStr">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="M19" s="9" t="inlineStr">
         <is>
-          <t>02_HUNIAN_ASRI_JATIHANDAP/01_Surat_Keluar/004_OT_YPL_03_IX_2026_Undangan_Open_Table_Pak_Fasha.pdf</t>
+          <t>02_HUNIAN_ASRI_JATIHANDAP/01_Surat_Keluar/005_OT_YPL_03_IX_2026_Undangan_Open_Table_Ibu_Re.pdf</t>
         </is>
       </c>
     </row>
@@ -1550,12 +1550,12 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>REG-2026-0015</t>
+          <t>REG-2026-0016</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>005/OT/YPL/03/IX/2026</t>
+          <t>006/OT/YPL/03/IX/2026</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -1585,12 +1585,12 @@
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>Undangan Open Table Jatihandap Asri di Dapur Hawu (Ibu Re)</t>
+          <t>Undangan Open Table Jatihandap Asri di Dapur Hawu (Pak Gun Gun)</t>
         </is>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>Ibu Re</t>
+          <t>Pak Gun Gun</t>
         </is>
       </c>
       <c r="K20" s="6" t="inlineStr">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="M20" s="6" t="inlineStr">
         <is>
-          <t>02_HUNIAN_ASRI_JATIHANDAP/01_Surat_Keluar/005_OT_YPL_03_IX_2026_Undangan_Open_Table_Ibu_Re.pdf</t>
+          <t>02_HUNIAN_ASRI_JATIHANDAP/01_Surat_Keluar/006_OT_YPL_03_IX_2026_Undangan_Open_Table_Pak_Gun_Gun.pdf</t>
         </is>
       </c>
     </row>
@@ -1615,12 +1615,12 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>REG-2026-0016</t>
+          <t>REG-2026-0017</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>006/OT/YPL/03/IX/2026</t>
+          <t>007/OT/YPL/03/IX/2026</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
@@ -1650,12 +1650,12 @@
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t>Undangan Open Table Jatihandap Asri di Dapur Hawu (Pak Gun Gun)</t>
+          <t>Undangan Open Table Jatihandap Asri di Dapur Hawu (Ibu Leni)</t>
         </is>
       </c>
       <c r="J21" s="9" t="inlineStr">
         <is>
-          <t>Pak Gun Gun</t>
+          <t>Ibu Leni</t>
         </is>
       </c>
       <c r="K21" s="9" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="M21" s="9" t="inlineStr">
         <is>
-          <t>02_HUNIAN_ASRI_JATIHANDAP/01_Surat_Keluar/006_OT_YPL_03_IX_2026_Undangan_Open_Table_Pak_Gun_Gun.pdf</t>
+          <t>02_HUNIAN_ASRI_JATIHANDAP/01_Surat_Keluar/007_OT_YPL_03_IX_2026_Undangan_Open_Table_Ibu_Leni.pdf</t>
         </is>
       </c>
     </row>
@@ -1680,12 +1680,12 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>REG-2026-0017</t>
+          <t>REG-2026-0018</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>007/OT/YPL/03/IX/2026</t>
+          <t>008/OT/YPL/03/IX/2026</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -1715,12 +1715,12 @@
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>Undangan Open Table Jatihandap Asri di Dapur Hawu (Ibu Leni)</t>
+          <t>Undangan Open Table Jatihandap Asri di Dapur Hawu (Pak Tomi)</t>
         </is>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
-          <t>Ibu Leni</t>
+          <t>Pak Tomi</t>
         </is>
       </c>
       <c r="K22" s="6" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="M22" s="6" t="inlineStr">
         <is>
-          <t>02_HUNIAN_ASRI_JATIHANDAP/01_Surat_Keluar/007_OT_YPL_03_IX_2026_Undangan_Open_Table_Ibu_Leni.pdf</t>
+          <t>02_HUNIAN_ASRI_JATIHANDAP/01_Surat_Keluar/008_OT_YPL_03_IX_2026_Undangan_Open_Table_Pak_Tomi.pdf</t>
         </is>
       </c>
     </row>
@@ -1745,12 +1745,12 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>REG-2026-0018</t>
+          <t>REG-2026-0019</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>008/OT/YPL/03/IX/2026</t>
+          <t>009/OT/YPL/03/IX/2026</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -1780,12 +1780,12 @@
       </c>
       <c r="I23" s="9" t="inlineStr">
         <is>
-          <t>Undangan Open Table Jatihandap Asri di Dapur Hawu (Pak Tomi)</t>
+          <t>Undangan Open Table Jatihandap Asri di Dapur Hawu (Pak Gilang)</t>
         </is>
       </c>
       <c r="J23" s="9" t="inlineStr">
         <is>
-          <t>Pak Tomi</t>
+          <t>Pak Gilang</t>
         </is>
       </c>
       <c r="K23" s="9" t="inlineStr">
@@ -1800,7 +1800,7 @@
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>02_HUNIAN_ASRI_JATIHANDAP/01_Surat_Keluar/008_OT_YPL_03_IX_2026_Undangan_Open_Table_Pak_Tomi.pdf</t>
+          <t>02_HUNIAN_ASRI_JATIHANDAP/01_Surat_Keluar/009_OT_YPL_03_IX_2026_Undangan_Open_Table_Pak_Gilang.pdf</t>
         </is>
       </c>
     </row>
@@ -1810,12 +1810,12 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>REG-2026-0019</t>
+          <t>REG-2026-0020</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>009/OT/YPL/03/IX/2026</t>
+          <t>010/OT/YPL/03/IX/2026</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -1845,12 +1845,12 @@
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>Undangan Open Table Jatihandap Asri di Dapur Hawu (Pak Gilang)</t>
+          <t>Undangan Open Table Jatihandap Asri di Dapur Hawu (Bu Mey)</t>
         </is>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
-          <t>Pak Gilang</t>
+          <t>Bu Mey</t>
         </is>
       </c>
       <c r="K24" s="6" t="inlineStr">
@@ -1865,7 +1865,7 @@
       </c>
       <c r="M24" s="6" t="inlineStr">
         <is>
-          <t>02_HUNIAN_ASRI_JATIHANDAP/01_Surat_Keluar/009_OT_YPL_03_IX_2026_Undangan_Open_Table_Pak_Gilang.pdf</t>
+          <t>02_HUNIAN_ASRI_JATIHANDAP/01_Surat_Keluar/010_OT_YPL_03_IX_2026_Undangan_Open_Table_Bu_Mey.pdf</t>
         </is>
       </c>
     </row>
@@ -1875,12 +1875,12 @@
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>REG-2026-0020</t>
+          <t>REG-2026-0021</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>010/OT/YPL/03/IX/2026</t>
+          <t>011/OT/YPL/03/IX/2026</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
@@ -1910,12 +1910,12 @@
       </c>
       <c r="I25" s="9" t="inlineStr">
         <is>
-          <t>Undangan Open Table Jatihandap Asri di Dapur Hawu (Bu Mey)</t>
+          <t>Undangan Open Table Jatihandap Asri di Dapur Hawu (Bu Haunurida)</t>
         </is>
       </c>
       <c r="J25" s="9" t="inlineStr">
         <is>
-          <t>Bu Mey</t>
+          <t>Bu Haunurida</t>
         </is>
       </c>
       <c r="K25" s="9" t="inlineStr">
@@ -1930,7 +1930,7 @@
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>02_HUNIAN_ASRI_JATIHANDAP/01_Surat_Keluar/010_OT_YPL_03_IX_2026_Undangan_Open_Table_Bu_Mey.pdf</t>
+          <t>02_HUNIAN_ASRI_JATIHANDAP/01_Surat_Keluar/011_OT_YPL_03_IX_2026_Undangan_Open_Table_Bu_Haunurida.pdf</t>
         </is>
       </c>
     </row>
@@ -1940,52 +1940,52 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>REG-2026-0021</t>
+          <t>REG-2026-0022</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>011/OT/YPL/03/IX/2026</t>
+          <t>021/SAB-DIR/EXT/VIII/2026</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>HJA</t>
+          <t>CORP</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>YPL</t>
+          <t>SAB</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>MKT</t>
+          <t>DIR</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>UNDANGAN</t>
+          <t>SURAT_KELUAR</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>Undangan Open Table Jatihandap Asri di Dapur Hawu (Bu Haunurida)</t>
+          <t>Surat Pemberitahuan Izin Tinggal &amp; Delegasi Hunian Sementara Majesty Apartment</t>
         </is>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>Bu Haunurida</t>
+          <t>Badan Pengelola Majesty Apartment Bandung</t>
         </is>
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t>Tim Marketing Jatihandap Asri</t>
+          <t>Direktur Utama PT SAB (Bpk. Yana Priatna)</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr">
@@ -1995,7 +1995,7 @@
       </c>
       <c r="M26" s="6" t="inlineStr">
         <is>
-          <t>02_HUNIAN_ASRI_JATIHANDAP/01_Surat_Keluar/011_OT_YPL_03_IX_2026_Undangan_Open_Table_Bu_Haunurida.pdf</t>
+          <t>07_CORPORATE_YANPROLAND_HOLDING/02_Surat_Tugas_Dan_Kuasa/021_SAB_DIR_EXT_VIII_2026_Surat_Pemberitahuan_Izin_Tinggal_Majesty_732.docx</t>
         </is>
       </c>
     </row>
@@ -2005,52 +2005,52 @@
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>REG-2026-0022</t>
+          <t>REG-2026-0023</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>021/SAB-DIR/EXT/VIII/2026</t>
+          <t>[PKS-KAB-2026-07-20]</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>CORP</t>
+          <t>GREN</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>SAB</t>
+          <t>KAB</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>DIR</t>
+          <t>MKT</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>SURAT_KELUAR</t>
+          <t>SPK</t>
         </is>
       </c>
       <c r="I27" s="9" t="inlineStr">
         <is>
-          <t>Surat Pemberitahuan Izin Tinggal &amp; Delegasi Hunian Sementara Majesty Apartment</t>
+          <t>PKS Optimalisasi Lead Gen &amp; Coaching Digital Marketing (Aswar Anas)</t>
         </is>
       </c>
       <c r="J27" s="9" t="inlineStr">
         <is>
-          <t>Badan Pengelola Majesty Apartment Bandung</t>
+          <t>Aswar Anas</t>
         </is>
       </c>
       <c r="K27" s="9" t="inlineStr">
         <is>
-          <t>Direktur Utama PT SAB (Bpk. Yana Priatna)</t>
+          <t>PT Kenzo Anatha Bumi (Yana Priatna)</t>
         </is>
       </c>
       <c r="L27" s="7" t="inlineStr">
@@ -2060,7 +2060,7 @@
       </c>
       <c r="M27" s="9" t="inlineStr">
         <is>
-          <t>07_CORPORATE_YANPROLAND_HOLDING/02_Surat_Tugas_Dan_Kuasa/021_SAB_DIR_EXT_VIII_2026_Surat_Pemberitahuan_Izin_Tinggal_Majesty_732.docx</t>
+          <t>01_GREN_PROPERTYKOST/06_SPK_Dan_Kontrak/PKS_PT_Kenzo_Anatha_Bumi_Aswar_Anas_Digital_Marketing_Meta_Ads.docx</t>
         </is>
       </c>
     </row>
@@ -2075,12 +2075,12 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>[PKS-KAB-2026-07-20]</t>
+          <t>004/MKT/KAB/GREN/IX/2026</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -2100,97 +2100,32 @@
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>SPK</t>
+          <t>IOM</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>PKS Optimalisasi Lead Gen &amp; Coaching Digital Marketing (Aswar Anas)</t>
+          <t>Kebijakan Program Penjualan &amp; Aktivasi Marketing Kuartal IV 2026</t>
         </is>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>Aswar Anas</t>
+          <t>Divisi Sales &amp; Marketing GREN Propertykost</t>
         </is>
       </c>
       <c r="K28" s="6" t="inlineStr">
         <is>
-          <t>PT Kenzo Anatha Bumi (Yana Priatna)</t>
+          <t>Divisi Marketing Communication</t>
         </is>
       </c>
       <c r="L28" s="4" t="inlineStr">
         <is>
-          <t>TERARSIP</t>
+          <t>DITERBITKAN</t>
         </is>
       </c>
       <c r="M28" s="6" t="inlineStr">
         <is>
-          <t>01_GREN_PROPERTYKOST/06_SPK_Dan_Kontrak/PKS_PT_Kenzo_Anatha_Bumi_Aswar_Anas_Digital_Marketing_Meta_Ads.docx</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="24" customHeight="1">
-      <c r="A29" s="7" t="n">
-        <v>24</v>
-      </c>
-      <c r="B29" s="8" t="inlineStr">
-        <is>
-          <t>REG-2026-0024</t>
-        </is>
-      </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>005/MKT/KAB/GREN/IX/2026</t>
-        </is>
-      </c>
-      <c r="D29" s="7" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="inlineStr">
-        <is>
-          <t>GREN</t>
-        </is>
-      </c>
-      <c r="F29" s="7" t="inlineStr">
-        <is>
-          <t>KAB</t>
-        </is>
-      </c>
-      <c r="G29" s="7" t="inlineStr">
-        <is>
-          <t>MKT</t>
-        </is>
-      </c>
-      <c r="H29" s="7" t="inlineStr">
-        <is>
-          <t>IOM</t>
-        </is>
-      </c>
-      <c r="I29" s="9" t="inlineStr">
-        <is>
-          <t>Kebijakan Program Penjualan &amp; Aktivasi Marketing Kuartal IV 2026</t>
-        </is>
-      </c>
-      <c r="J29" s="9" t="inlineStr">
-        <is>
-          <t>Divisi Sales &amp; Marketing GREN Propertykost</t>
-        </is>
-      </c>
-      <c r="K29" s="9" t="inlineStr">
-        <is>
-          <t>Divisi Marketing Communication</t>
-        </is>
-      </c>
-      <c r="L29" s="7" t="inlineStr">
-        <is>
-          <t>DITERBITKAN</t>
-        </is>
-      </c>
-      <c r="M29" s="9" t="inlineStr">
-        <is>
-          <t>01_GREN_PROPERTYKOST/03_Internal_Office_Memo_IOM/005_MKT_KAB_GREN_IX_2026_IOM_Program_Penjualan_Sales.docx</t>
+          <t>01_GREN_PROPERTYKOST/03_Internal_Office_Memo_IOM/004_MKT_KAB_GREN_IX_2026_IOM_Program_Penjualan_Sales.docx</t>
         </is>
       </c>
     </row>
@@ -2925,7 +2860,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Total Dokumen Terdaftar: 24 Berkas</t>
+          <t>Total Dokumen Terdaftar: 23 Berkas</t>
         </is>
       </c>
     </row>
@@ -2971,11 +2906,11 @@
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>33.3%</t>
+          <t>30.4%</t>
         </is>
       </c>
     </row>
@@ -2998,7 +2933,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>45.8%</t>
+          <t>47.8%</t>
         </is>
       </c>
     </row>
@@ -3067,7 +3002,7 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>4.2%</t>
+          <t>4.3%</t>
         </is>
       </c>
     </row>
@@ -3113,7 +3048,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>17.4%</t>
         </is>
       </c>
     </row>
@@ -3130,7 +3065,7 @@
         </is>
       </c>
       <c r="D12" s="14" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: terbitkan IOM resmi PT KAB No. 004/MKT/KAB/GREN/IX/2026 Kebijakan Fee Rukost 10% Cash Keras 21 Hari
</commit_message>
<xml_diff>
--- a/00_STANDAR_DAN_REGULASI/BUKU_AGENDA_DAN_REGISTER_NOMOR_SURAT.xlsx
+++ b/00_STANDAR_DAN_REGULASI/BUKU_AGENDA_DAN_REGISTER_NOMOR_SURAT.xlsx
@@ -2105,17 +2105,17 @@
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>Kebijakan Program Penjualan &amp; Aktivasi Marketing Kuartal IV 2026</t>
+          <t>Kebijakan Skema Fee Penjualan Rukost 10% Cash Keras (Masa Berlaku 21 Hari)</t>
         </is>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>Divisi Sales &amp; Marketing GREN Propertykost</t>
+          <t>Seluruh Rekan Sales &amp; Agent (All Team)</t>
         </is>
       </c>
       <c r="K28" s="6" t="inlineStr">
         <is>
-          <t>Divisi Marketing Communication</t>
+          <t>Nugi Fathul Falah (SPV Markom &amp; Digital)</t>
         </is>
       </c>
       <c r="L28" s="4" t="inlineStr">
@@ -2125,7 +2125,7 @@
       </c>
       <c r="M28" s="6" t="inlineStr">
         <is>
-          <t>01_GREN_PROPERTYKOST/03_Internal_Office_Memo_IOM/004_MKT_KAB_GREN_IX_2026_IOM_Program_Penjualan_Sales.docx</t>
+          <t>01_GREN_PROPERTYKOST/03_Internal_Office_Memo_IOM/004_MKT_KAB_GREN_IX_2026_IOM_Skema_Fee_Rukost_Cash_Keras_10_Persen.docx</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: batasi ruang lingkup IOM No. 004 khusus Tim Sales Marketing (tanpa agent freelance/rekanan)
</commit_message>
<xml_diff>
--- a/00_STANDAR_DAN_REGULASI/BUKU_AGENDA_DAN_REGISTER_NOMOR_SURAT.xlsx
+++ b/00_STANDAR_DAN_REGULASI/BUKU_AGENDA_DAN_REGISTER_NOMOR_SURAT.xlsx
@@ -2105,12 +2105,12 @@
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>Kebijakan Skema Fee Penjualan Rukost 10% Cash Keras (Masa Berlaku 21 Hari)</t>
+          <t>Kebijakan Skema Fee Penjualan Rukost 10% Khusus Cash Keras (Tim Sales Marketing)</t>
         </is>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>Seluruh Rekan Sales &amp; Agent (All Team)</t>
+          <t>Seluruh Rekan Tim Sales &amp; Marketing GREN Propertykost</t>
         </is>
       </c>
       <c r="K28" s="6" t="inlineStr">

</xml_diff>

<commit_message>
docs(register): update master Excel, CSV, and JSON registers with latest Direktur Utama IOM 004
</commit_message>
<xml_diff>
--- a/00_STANDAR_DAN_REGULASI/BUKU_AGENDA_DAN_REGISTER_NOMOR_SURAT.xlsx
+++ b/00_STANDAR_DAN_REGULASI/BUKU_AGENDA_DAN_REGISTER_NOMOR_SURAT.xlsx
@@ -562,11 +562,10 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Terakhir Diperbarui: 21 September 2026 | Total Terdaftar: 23 Berkas</t>
-        </is>
-      </c>
-    </row>
-    <row r="4"/>
+          <t>Terakhir Diperbarui: 21 September 2026 | Total Terdaftar: 24 Berkas</t>
+        </is>
+      </c>
+    </row>
     <row r="5" ht="28" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -2105,7 +2104,7 @@
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>Kebijakan Skema Fee Penjualan Rukost 10% Khusus Cash Keras (Tim Sales Marketing)</t>
+          <t>Kebijakan Skema Fee Penjualan Rukost 10% Khusus Cash Keras 21 Hari (Tim Sales Marketing)</t>
         </is>
       </c>
       <c r="J28" s="6" t="inlineStr">
@@ -2115,17 +2114,17 @@
       </c>
       <c r="K28" s="6" t="inlineStr">
         <is>
-          <t>Nugi Fathul Falah (SPV Markom &amp; Digital)</t>
+          <t>Direktur Utama PT. Kenzo Anatha Bumi (Bapak Yana Priatna)</t>
         </is>
       </c>
       <c r="L28" s="4" t="inlineStr">
         <is>
-          <t>DITERBITKAN</t>
+          <t>DITERBITKAN &amp; DITANDATANGANI</t>
         </is>
       </c>
       <c r="M28" s="6" t="inlineStr">
         <is>
-          <t>01_GREN_PROPERTYKOST/03_Internal_Office_Memo_IOM/004_MKT_KAB_GREN_IX_2026_IOM_Skema_Fee_Rukost_Cash_Keras_10_Persen.docx</t>
+          <t>01_GREN_PROPERTYKOST/03_Internal_Office_Memo_IOM/004_MKT_KAB_GREN_IX_2026_IOM_Skema_Fee_Rukost_Cash_Keras_10_Persen.docx (dan .pdf)</t>
         </is>
       </c>
     </row>

</xml_diff>